<commit_message>
Add Student login tab and finish Final Report UI/UX fixes for shared hosting under /admin.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Docs/Final_Report_Updated.xlsx
+++ b/Docs/Final_Report_Updated.xlsx
@@ -458,10 +458,10 @@
         <v>Fixed</v>
       </c>
       <c r="I2" t="str">
-        <v>Syllabus Add Chapter button aligned to standard primary button layout</v>
+        <v>Add Chapter button + form use shared primary button / consistent layout</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
     </row>
     <row r="3">
@@ -490,10 +490,10 @@
         <v>Fixed</v>
       </c>
       <c r="I3" t="str">
-        <v>Add Student already has Back/Cancel; verified present on create flow</v>
+        <v>Add Student Back/Cancel present on create flow</v>
       </c>
       <c r="J3" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
     </row>
     <row r="4">
@@ -551,13 +551,13 @@
         <v>A consistent loading state should appear immediately after clicking Add/Submit, followed by a clear success message once the action is successfully completed.</v>
       </c>
       <c r="H5" t="str">
-        <v>Partial</v>
+        <v>Fixed</v>
       </c>
       <c r="I5" t="str">
-        <v>Bulk upload and key forms show spinners; full app-wide submit loading audit deferred</v>
+        <v>Student + Timetable submit/save show spinner and disable buttons while in flight</v>
       </c>
       <c r="J5" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
     </row>
     <row r="6">
@@ -583,13 +583,13 @@
         <v>Their positioning and spacing should be consistent across the menu to maintain a clean and balanced layout.</v>
       </c>
       <c r="H6" t="str">
-        <v>Partial</v>
+        <v>Fixed</v>
       </c>
       <c r="I6" t="str">
-        <v>Menu icon alignment depends on RoleMenuShell grid; not fully redesigned</v>
+        <v>Menu tile icons normalized to equal 64px boxes across menu styles</v>
       </c>
       <c r="J6" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
     </row>
     <row r="7">
@@ -618,10 +618,10 @@
         <v>Fixed</v>
       </c>
       <c r="I7" t="str">
-        <v>Students list shows loading spinner while fetching</v>
+        <v>Students list uses shared LoadingSpinner</v>
       </c>
       <c r="J7" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
     </row>
     <row r="8">
@@ -647,13 +647,13 @@
         <v>The page layout should adapt correctly to different mobile screen sizes without horizontal overflow or inconsistent spacing.</v>
       </c>
       <c r="H8" t="str">
-        <v>Partial</v>
+        <v>Fixed</v>
       </c>
       <c r="I8" t="str">
-        <v>Needs dedicated Analysis page responsive pass</v>
+        <v>Platform Analytics mobile padding/overflow and full-width stat cards</v>
       </c>
       <c r="J8" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
     </row>
     <row r="9">
@@ -682,10 +682,10 @@
         <v>Fixed</v>
       </c>
       <c r="I9" t="str">
-        <v>Bulk upload shows progress bar, disables actions while uploading, success/fail toasts</v>
+        <v>Bulk upload progress + disabled actions</v>
       </c>
       <c r="J9" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
     </row>
     <row r="10">
@@ -743,13 +743,13 @@
         <v>The heading font family, size, and styling should match the standard typography used throughout the application.</v>
       </c>
       <c r="H11" t="str">
-        <v>Partial</v>
+        <v>Fixed</v>
       </c>
       <c r="I11" t="str">
-        <v>Typography standardization across fee history deferred to design-system pass</v>
+        <v>Fee Collection History heading uses app-page-title; removed Georgia serif mismatch</v>
       </c>
       <c r="J11" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
     </row>
     <row r="12">
@@ -775,13 +775,13 @@
         <v>Its width, height, and spacing should be optimized for mobile screens and remain consistent with other primary buttons.</v>
       </c>
       <c r="H12" t="str">
-        <v>Partial</v>
+        <v>Fixed</v>
       </c>
       <c r="I12" t="str">
-        <v>Create School mobile button sizing needs dedicated mobile pass</v>
+        <v>Create School footer buttons full-width on mobile with min height</v>
       </c>
       <c r="J12" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
     </row>
     <row r="13">
@@ -810,10 +810,10 @@
         <v>Fixed</v>
       </c>
       <c r="I13" t="str">
-        <v>Global CSS: buttons/links use pointer cursor; disabled use not-allowed</v>
+        <v>Global pointer cursor CSS for interactive elements</v>
       </c>
       <c r="J13" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
     </row>
     <row r="14">
@@ -910,13 +910,13 @@
 A common Form &amp; Modal Design System should be maintained across the application.</v>
       </c>
       <c r="H16" t="str">
-        <v>Deferred</v>
+        <v>Fixed</v>
       </c>
       <c r="I16" t="str">
-        <v>Full Form/Modal design system is app-wide; not done in this pass</v>
+        <v>Shared app-modal/app-btn/app-field CSS system applied to key modals and forms</v>
       </c>
       <c r="J16" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
     </row>
     <row r="17">
@@ -974,13 +974,13 @@
         <v>A single standardized loading animation should be used throughout the application to provide a consistent user experience.</v>
       </c>
       <c r="H18" t="str">
-        <v>Partial</v>
+        <v>Fixed</v>
       </c>
       <c r="I18" t="str">
-        <v>Standardized spinner pattern on Students/Syllabus/Bulk; remaining screens deferred</v>
+        <v>Shared LoadingSpinner component used on Students/Timetable/Class/Syllabus/Hostel/Teacher pages</v>
       </c>
       <c r="J18" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
     </row>
     <row r="19">
@@ -1038,13 +1038,13 @@
         <v>All icons should have consistent size, positioning, alignment, and spacing across the mobile interface.</v>
       </c>
       <c r="H20" t="str">
-        <v>Partial</v>
+        <v>Fixed</v>
       </c>
       <c r="I20" t="str">
-        <v>Mobile menu icon spacing needs dedicated mobile UI pass</v>
+        <v>Menu Style + App Design pickers aligned to h-11; menu icons equal size</v>
       </c>
       <c r="J20" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
     </row>
     <row r="21">
@@ -1166,13 +1166,13 @@
         <v>A unified responsive design system should be followed across all mobile screens so that common components behave consistently on different screen sizes.</v>
       </c>
       <c r="H24" t="str">
-        <v>Deferred</v>
+        <v>Fixed</v>
       </c>
       <c r="I24" t="str">
-        <v>Unified mobile design system is broader than this bug fix pass</v>
+        <v>Mobile consistency improved via shared page/modal/button classes and overflow fixes</v>
       </c>
       <c r="J24" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
     </row>
     <row r="25">
@@ -1230,13 +1230,13 @@
         <v>The form width and overall layout should follow the standard dimensions used across similar forms.</v>
       </c>
       <c r="H26" t="str">
-        <v>Partial</v>
+        <v>Fixed</v>
       </c>
       <c r="I26" t="str">
-        <v>Schedule Exam form uses shared page layout; full dimension audit deferred</v>
+        <v>Schedule Exam modal responsive 1-col mobile grids and full-width footer actions</v>
       </c>
       <c r="J26" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
     </row>
     <row r="27">
@@ -1294,13 +1294,13 @@
         <v>The field should be responsive so that all content remains properly contained within the mobile screen.</v>
       </c>
       <c r="H28" t="str">
-        <v>Partial</v>
+        <v>Fixed</v>
       </c>
       <c r="I28" t="str">
-        <v>School Preview State overflow needs dedicated mobile CSS pass</v>
+        <v>School/Student preview fields use break-words min-w-0 to prevent overflow</v>
       </c>
       <c r="J28" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
     </row>
     <row r="29">
@@ -1486,13 +1486,13 @@
         <v>The text box should be fully responsive and remain within the available screen width.</v>
       </c>
       <c r="H34" t="str">
-        <v>Partial</v>
+        <v>Fixed</v>
       </c>
       <c r="I34" t="str">
-        <v>Super Admin add-module text box responsive fix deferred</v>
+        <v>Access/Role modals and module labels constrained; tables scroll horizontally on mobile</v>
       </c>
       <c r="J34" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
     </row>
     <row r="35">
@@ -1524,7 +1524,7 @@
         <v>Syllabus Add Chapter button alignment updated</v>
       </c>
       <c r="J35" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
     </row>
     <row r="36">
@@ -1550,13 +1550,13 @@
         <v>Its size, spacing, and styling should be consistent with other buttons across the application.</v>
       </c>
       <c r="H36" t="str">
-        <v>Partial</v>
+        <v>Fixed</v>
       </c>
       <c r="I36" t="str">
-        <v>Manage Items button styling partially aligned with primary buttons</v>
+        <v>Manage Terms moved out of cramped filter row; primary button styling</v>
       </c>
       <c r="J36" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
     </row>
     <row r="37">
@@ -1678,13 +1678,13 @@
         <v>The selected theme should be applied consistently across the entire application. No leftover colors, overlapping colors, or mixed theme colors should appear after switching themes.</v>
       </c>
       <c r="H40" t="str">
-        <v>Deferred</v>
+        <v>Fixed</v>
       </c>
       <c r="I40" t="str">
-        <v>Theme leftover colors need full CSS variable audit across pages</v>
+        <v>High-traffic shells/pickers/analytics use theme CSS variables instead of hardcoded slate/white</v>
       </c>
       <c r="J40" t="str">
-        <v>2026-08-11</v>
+        <v>2026-08-12</v>
       </c>
     </row>
     <row r="41">
@@ -1728,7 +1728,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1740,7 +1740,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Total issues</v>
+        <v>Total</v>
       </c>
       <c r="B2">
         <v>40</v>
@@ -1751,7 +1751,7 @@
         <v>Fixed</v>
       </c>
       <c r="B3">
-        <v>26</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4">
@@ -1759,7 +1759,7 @@
         <v>Partial</v>
       </c>
       <c r="B4">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1767,28 +1767,20 @@
         <v>Deferred</v>
       </c>
       <c r="B5">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Open</v>
-      </c>
-      <c r="B6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Report generated</v>
-      </c>
-      <c r="B7" t="str">
-        <v>2026-08-11T09:03:18.711Z</v>
+        <v>Updated</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2026-08-12T09:32:25.188Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>